<commit_message>
adjusted parametrization for reference simulation but didn't check after imposing seminal & adventitious emergence
</commit_message>
<xml_diff>
--- a/simulations/inputs/Scenarios_24_05.xlsx
+++ b/simulations/inputs/Scenarios_24_05.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tigerault\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp14043\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{545148BC-01FF-42D2-954E-3A567E88CE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B28F8671-BAE9-4741-A5A4-E8B860609B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios_as_columns" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1984" uniqueCount="577">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1985" uniqueCount="578">
   <si>
     <t>input_file</t>
   </si>
@@ -1765,6 +1765,9 @@
   </si>
   <si>
     <t>Maximal rate of amino acid synthesis in the root segment</t>
+  </si>
+  <si>
+    <t>confirm</t>
   </si>
 </sst>
 </file>
@@ -2632,48 +2635,48 @@
     </xf>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20 % - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
     <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
     <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
     <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
     <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
     <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Avertissement" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Calcul" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Cellule liée" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Entrée" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Insatisfaisant" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Neutre" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Satisfaisant" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Sortie" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Texte explicatif" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Titre" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Titre 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Titre 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Titre 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Titre 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Vérification" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2951,18 +2954,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M232"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M233"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" style="1" customWidth="1"/>
     <col min="2" max="4" width="15" style="1" customWidth="1"/>
-    <col min="5" max="5" width="58.140625" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" customWidth="1"/>
-    <col min="7" max="7" width="19.5703125" style="37" customWidth="1"/>
-    <col min="8" max="13" width="39.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="58.109375" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19.5546875" style="37" customWidth="1"/>
+    <col min="8" max="13" width="39.88671875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>469</v>
       </c>
@@ -3003,7 +3006,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>540</v>
       </c>
@@ -3044,7 +3047,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>472</v>
       </c>
@@ -3085,7 +3088,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="4" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>484</v>
       </c>
@@ -3126,7 +3129,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="5" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>483</v>
       </c>
@@ -3167,7 +3170,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="6" spans="1:13" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>490</v>
       </c>
@@ -3208,7 +3211,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>485</v>
       </c>
@@ -3249,7 +3252,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="8" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>545</v>
       </c>
@@ -3290,7 +3293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -3331,7 +3334,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>3</v>
       </c>
@@ -3372,7 +3375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="74" t="s">
         <v>444</v>
       </c>
@@ -3413,7 +3416,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>4</v>
       </c>
@@ -3454,7 +3457,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>5</v>
       </c>
@@ -3495,7 +3498,7 @@
         <v>4.1666666999999998E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>20</v>
       </c>
@@ -3536,7 +3539,7 @@
         <v>4.1666666999999998E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>1</v>
       </c>
@@ -3577,7 +3580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>448</v>
       </c>
@@ -3618,7 +3621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>6</v>
       </c>
@@ -3659,7 +3662,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>7</v>
       </c>
@@ -3700,7 +3703,7 @@
         <v>5.0000000000000001E-9</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>8</v>
       </c>
@@ -3741,7 +3744,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>461</v>
       </c>
@@ -3782,7 +3785,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>462</v>
       </c>
@@ -3823,7 +3826,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>465</v>
       </c>
@@ -3864,7 +3867,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>467</v>
       </c>
@@ -3905,7 +3908,7 @@
         <v>86400</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
         <v>10</v>
       </c>
@@ -3946,7 +3949,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
         <v>11</v>
       </c>
@@ -3987,7 +3990,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>363</v>
       </c>
@@ -4028,7 +4031,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
         <v>365</v>
       </c>
@@ -4069,7 +4072,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
         <v>377</v>
       </c>
@@ -4110,7 +4113,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>376</v>
       </c>
@@ -4151,7 +4154,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>375</v>
       </c>
@@ -4192,7 +4195,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>12</v>
       </c>
@@ -4233,7 +4236,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
         <v>13</v>
       </c>
@@ -4274,7 +4277,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="s">
         <v>14</v>
       </c>
@@ -4315,7 +4318,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
         <v>9</v>
       </c>
@@ -4356,7 +4359,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>454</v>
       </c>
@@ -4397,7 +4400,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="13" t="s">
         <v>21</v>
       </c>
@@ -4438,7 +4441,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" s="13" t="s">
         <v>22</v>
       </c>
@@ -4479,7 +4482,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="13" t="s">
         <v>23</v>
       </c>
@@ -4520,7 +4523,7 @@
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" s="13" t="s">
         <v>24</v>
       </c>
@@ -4561,7 +4564,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
         <v>25</v>
       </c>
@@ -4602,7 +4605,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="13" t="s">
         <v>26</v>
       </c>
@@ -4643,7 +4646,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" s="13" t="s">
         <v>27</v>
       </c>
@@ -4684,7 +4687,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" s="13" t="s">
         <v>28</v>
       </c>
@@ -4725,7 +4728,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="13" t="s">
         <v>29</v>
       </c>
@@ -4766,7 +4769,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="13" t="s">
         <v>30</v>
       </c>
@@ -4807,7 +4810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" s="13" t="s">
         <v>31</v>
       </c>
@@ -4848,7 +4851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" s="13" t="s">
         <v>32</v>
       </c>
@@ -4889,7 +4892,7 @@
         <v>-0.1</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" s="13" t="s">
         <v>33</v>
       </c>
@@ -4930,7 +4933,7 @@
         <v>-0.2</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" s="13" t="s">
         <v>34</v>
       </c>
@@ -4971,7 +4974,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" s="13" t="s">
         <v>35</v>
       </c>
@@ -5012,7 +5015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" s="13" t="s">
         <v>434</v>
       </c>
@@ -5053,7 +5056,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" s="13" t="s">
         <v>435</v>
       </c>
@@ -5094,7 +5097,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" s="13" t="s">
         <v>457</v>
       </c>
@@ -5135,7 +5138,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" s="13" t="s">
         <v>15</v>
       </c>
@@ -5176,7 +5179,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" s="11" t="s">
         <v>16</v>
       </c>
@@ -5217,7 +5220,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" s="11" t="s">
         <v>17</v>
       </c>
@@ -5258,7 +5261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" s="11" t="s">
         <v>18</v>
       </c>
@@ -5299,7 +5302,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" s="11" t="s">
         <v>19</v>
       </c>
@@ -5340,7 +5343,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" s="15" t="s">
         <v>36</v>
       </c>
@@ -5381,7 +5384,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" s="15" t="s">
         <v>380</v>
       </c>
@@ -5422,7 +5425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" s="15" t="s">
         <v>37</v>
       </c>
@@ -5463,7 +5466,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" s="15" t="s">
         <v>38</v>
       </c>
@@ -5504,7 +5507,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" s="17" t="s">
         <v>39</v>
       </c>
@@ -5545,7 +5548,7 @@
         <v>6.9999999999999999E-4</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" s="17" t="s">
         <v>40</v>
       </c>
@@ -5586,7 +5589,7 @@
         <v>1.22E-4</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A65" s="17" t="s">
         <v>207</v>
       </c>
@@ -5627,7 +5630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A66" s="17" t="s">
         <v>41</v>
       </c>
@@ -5668,7 +5671,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A67" s="17" t="s">
         <v>406</v>
       </c>
@@ -5709,7 +5712,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A68" s="17" t="s">
         <v>91</v>
       </c>
@@ -5750,7 +5753,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A69" s="17" t="s">
         <v>408</v>
       </c>
@@ -5791,7 +5794,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A70" s="17" t="s">
         <v>42</v>
       </c>
@@ -5832,7 +5835,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A71" s="17" t="s">
         <v>208</v>
       </c>
@@ -5873,7 +5876,7 @@
         <v>1453890.8941884842</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" s="17" t="s">
         <v>43</v>
       </c>
@@ -5914,7 +5917,7 @@
         <v>1.3888888888888888E-5</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A73" s="17" t="s">
         <v>44</v>
       </c>
@@ -5955,7 +5958,7 @@
         <v>6.5011574074074071E-4</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A74" s="17" t="s">
         <v>45</v>
       </c>
@@ -5996,7 +5999,7 @@
         <v>4.7400000000000003E-3</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A75" s="17" t="s">
         <v>46</v>
       </c>
@@ -6037,7 +6040,7 @@
         <v>282528</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A76" s="17" t="s">
         <v>47</v>
       </c>
@@ -6078,7 +6081,7 @@
         <v>0.56999999999999995</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A77" s="17" t="s">
         <v>48</v>
       </c>
@@ -6119,7 +6122,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A78" s="17" t="s">
         <v>49</v>
       </c>
@@ -6160,7 +6163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A79" s="33" t="s">
         <v>50</v>
       </c>
@@ -6201,7 +6204,7 @@
         <v>745476480000</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A80" s="33" t="s">
         <v>205</v>
       </c>
@@ -6242,7 +6245,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" s="33" t="s">
         <v>414</v>
       </c>
@@ -6283,7 +6286,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" s="33" t="s">
         <v>400</v>
       </c>
@@ -6324,7 +6327,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" s="33" t="s">
         <v>410</v>
       </c>
@@ -6365,7 +6368,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" s="33" t="s">
         <v>401</v>
       </c>
@@ -6406,7 +6409,7 @@
         <v>60479.999999999993</v>
       </c>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" s="33" t="s">
         <v>411</v>
       </c>
@@ -6447,7 +6450,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" s="33" t="s">
         <v>402</v>
       </c>
@@ -6488,7 +6491,7 @@
         <v>518400</v>
       </c>
     </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" s="33" t="s">
         <v>412</v>
       </c>
@@ -6529,7 +6532,7 @@
         <v>5184000</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" s="17" t="s">
         <v>51</v>
       </c>
@@ -6570,7 +6573,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" s="17" t="s">
         <v>52</v>
       </c>
@@ -6611,7 +6614,7 @@
         <v>140000</v>
       </c>
     </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" s="17" t="s">
         <v>53</v>
       </c>
@@ -6652,7 +6655,7 @@
         <v>3.6636136999999999E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" s="17" t="s">
         <v>54</v>
       </c>
@@ -6693,7 +6696,7 @@
         <v>4.4999999999999997E-3</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" s="17" t="s">
         <v>55</v>
       </c>
@@ -6734,7 +6737,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A93" s="19" t="s">
         <v>214</v>
       </c>
@@ -6775,7 +6778,7 @@
         <v>6.0000000000000002E-6</v>
       </c>
     </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A94" s="19" t="s">
         <v>215</v>
       </c>
@@ -6816,7 +6819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A95" s="19" t="s">
         <v>216</v>
       </c>
@@ -6857,7 +6860,7 @@
         <v>374999999.99999994</v>
       </c>
     </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A96" s="19" t="s">
         <v>217</v>
       </c>
@@ -6898,7 +6901,7 @@
         <v>3.7037037037037038E-3</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A97" s="19" t="s">
         <v>218</v>
       </c>
@@ -6939,7 +6942,7 @@
         <v>165600</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A98" s="13" t="s">
         <v>60</v>
       </c>
@@ -6980,7 +6983,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A99" s="13" t="s">
         <v>209</v>
       </c>
@@ -7021,7 +7024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A100" s="13" t="s">
         <v>59</v>
       </c>
@@ -7062,7 +7065,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A101" s="23" t="s">
         <v>65</v>
       </c>
@@ -7103,7 +7106,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A102" s="23" t="s">
         <v>367</v>
       </c>
@@ -7144,7 +7147,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A103" s="23" t="s">
         <v>368</v>
       </c>
@@ -7185,7 +7188,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A104" s="23" t="s">
         <v>369</v>
       </c>
@@ -7226,7 +7229,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A105" s="23" t="s">
         <v>505</v>
       </c>
@@ -7267,7 +7270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A106" s="23" t="s">
         <v>385</v>
       </c>
@@ -7308,7 +7311,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A107" s="23" t="s">
         <v>506</v>
       </c>
@@ -7354,7 +7357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A108" s="23" t="s">
         <v>507</v>
       </c>
@@ -7400,7 +7403,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A109" s="23" t="s">
         <v>508</v>
       </c>
@@ -7446,7 +7449,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A110" s="23" t="s">
         <v>509</v>
       </c>
@@ -7492,7 +7495,7 @@
         <v>1470</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A111" s="23" t="s">
         <v>387</v>
       </c>
@@ -7533,7 +7536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A112" s="23" t="s">
         <v>389</v>
       </c>
@@ -7574,7 +7577,7 @@
         <v>1589759.9999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A113" s="23" t="s">
         <v>391</v>
       </c>
@@ -7615,7 +7618,7 @@
         <v>6171428.5714285718</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A114" s="23" t="s">
         <v>393</v>
       </c>
@@ -7656,7 +7659,7 @@
         <v>6171428.5714285718</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A115" s="23" t="s">
         <v>421</v>
       </c>
@@ -7697,7 +7700,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="116" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="23" t="s">
         <v>423</v>
       </c>
@@ -7743,7 +7746,7 @@
         <v>28080</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A117" s="23" t="s">
         <v>425</v>
       </c>
@@ -7789,7 +7792,7 @@
         <v>0.11100000000000002</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A118" s="23" t="s">
         <v>502</v>
       </c>
@@ -7830,7 +7833,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="119" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="23" t="s">
         <v>503</v>
       </c>
@@ -7876,7 +7879,7 @@
         <v>459648</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A120" s="23" t="s">
         <v>504</v>
       </c>
@@ -7922,7 +7925,7 @@
         <v>0.13875000000000001</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A121" s="23" t="s">
         <v>395</v>
       </c>
@@ -7963,7 +7966,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A122" s="23" t="s">
         <v>397</v>
       </c>
@@ -8004,7 +8007,7 @@
         <v>43200</v>
       </c>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A123" s="13" t="s">
         <v>61</v>
       </c>
@@ -8045,7 +8048,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A124" s="13" t="s">
         <v>62</v>
       </c>
@@ -8087,7 +8090,7 @@
         <v>2.0833333333333335E-4</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A125" s="13" t="s">
         <v>63</v>
       </c>
@@ -8128,7 +8131,7 @@
         <v>5.7899999999999998E-7</v>
       </c>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A126" s="13" t="s">
         <v>64</v>
       </c>
@@ -8169,7 +8172,7 @@
         <v>2.0833333333333335E-4</v>
       </c>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A127" s="13" t="s">
         <v>450</v>
       </c>
@@ -8210,7 +8213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A128" s="13" t="s">
         <v>452</v>
       </c>
@@ -8251,7 +8254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A129" s="68" t="s">
         <v>441</v>
       </c>
@@ -8296,7 +8299,7 @@
         <v>5.9999999999999997E-7</v>
       </c>
     </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A130" s="68" t="s">
         <v>67</v>
       </c>
@@ -8341,7 +8344,7 @@
         <v>8.3333333333333331E-5</v>
       </c>
     </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A131" s="68" t="s">
         <v>446</v>
       </c>
@@ -8382,7 +8385,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A132" s="21" t="s">
         <v>66</v>
       </c>
@@ -8423,7 +8426,7 @@
         <v>5.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A133" s="21" t="s">
         <v>438</v>
       </c>
@@ -8464,7 +8467,7 @@
         <v>4.9999999999999999E-13</v>
       </c>
     </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A134" s="21" t="s">
         <v>229</v>
       </c>
@@ -8505,7 +8508,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A135" s="21" t="s">
         <v>230</v>
       </c>
@@ -8546,7 +8549,7 @@
         <v>-0.04</v>
       </c>
     </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A136" s="21" t="s">
         <v>231</v>
       </c>
@@ -8587,7 +8590,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A137" s="21" t="s">
         <v>232</v>
       </c>
@@ -8628,7 +8631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A138" s="21" t="s">
         <v>68</v>
       </c>
@@ -8669,7 +8672,7 @@
         <v>1.9999999999999999E-7</v>
       </c>
     </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A139" s="21" t="s">
         <v>233</v>
       </c>
@@ -8710,7 +8713,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A140" s="21" t="s">
         <v>234</v>
       </c>
@@ -8751,7 +8754,7 @@
         <v>-0.04</v>
       </c>
     </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A141" s="21" t="s">
         <v>235</v>
       </c>
@@ -8792,7 +8795,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A142" s="21" t="s">
         <v>236</v>
       </c>
@@ -8833,7 +8836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A143" s="21" t="s">
         <v>69</v>
       </c>
@@ -8874,7 +8877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A144" s="72" t="s">
         <v>70</v>
       </c>
@@ -8915,7 +8918,7 @@
         <v>5.0000000000000004E-6</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A145" s="23" t="s">
         <v>56</v>
       </c>
@@ -8956,7 +8959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A146" s="23" t="s">
         <v>57</v>
       </c>
@@ -8997,7 +9000,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A147" s="23" t="s">
         <v>58</v>
       </c>
@@ -9038,7 +9041,7 @@
         <v>3.9999999999999998E-6</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A148" s="23" t="s">
         <v>71</v>
       </c>
@@ -9079,7 +9082,7 @@
         <v>3.7699999999999999E-10</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A149" s="23" t="s">
         <v>237</v>
       </c>
@@ -9120,7 +9123,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A150" s="23" t="s">
         <v>238</v>
       </c>
@@ -9161,7 +9164,7 @@
         <v>-0.06</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A151" s="23" t="s">
         <v>239</v>
       </c>
@@ -9202,7 +9205,7 @@
         <v>0.89100000000000001</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A152" s="23" t="s">
         <v>240</v>
       </c>
@@ -9243,7 +9246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A153" s="23" t="s">
         <v>72</v>
       </c>
@@ -9284,7 +9287,7 @@
         <v>4.0000000000000003E-5</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A154" s="13" t="s">
         <v>73</v>
       </c>
@@ -9325,7 +9328,7 @@
         <v>5.8333333333333335E-9</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A155" s="13" t="s">
         <v>241</v>
       </c>
@@ -9366,7 +9369,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A156" s="13" t="s">
         <v>242</v>
       </c>
@@ -9407,7 +9410,7 @@
         <v>-0.06</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A157" s="13" t="s">
         <v>243</v>
       </c>
@@ -9448,7 +9451,7 @@
         <v>0.89100000000000001</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A158" s="13" t="s">
         <v>244</v>
       </c>
@@ -9489,7 +9492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A159" s="13" t="s">
         <v>74</v>
       </c>
@@ -9530,7 +9533,7 @@
         <v>4.0000000000000003E-5</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A160" s="9" t="s">
         <v>75</v>
       </c>
@@ -9571,7 +9574,7 @@
         <v>4.0000000000000001E-8</v>
       </c>
     </row>
-    <row r="161" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A161" s="9" t="s">
         <v>219</v>
       </c>
@@ -9612,7 +9615,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="162" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A162" s="9" t="s">
         <v>220</v>
       </c>
@@ -9653,7 +9656,7 @@
         <v>-4.4200000000000003E-2</v>
       </c>
     </row>
-    <row r="163" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A163" s="9" t="s">
         <v>221</v>
       </c>
@@ -9694,7 +9697,7 @@
         <v>1.55</v>
       </c>
     </row>
-    <row r="164" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A164" s="9" t="s">
         <v>222</v>
       </c>
@@ -9735,7 +9738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A165" s="9" t="s">
         <v>76</v>
       </c>
@@ -9776,7 +9779,7 @@
         <v>2.7799999999999998E-4</v>
       </c>
     </row>
-    <row r="166" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A166" s="25" t="s">
         <v>78</v>
       </c>
@@ -9820,7 +9823,7 @@
         <v>2.4999999999999998E-12</v>
       </c>
     </row>
-    <row r="167" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A167" s="25" t="s">
         <v>246</v>
       </c>
@@ -9861,7 +9864,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="168" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A168" s="25" t="s">
         <v>247</v>
       </c>
@@ -9902,7 +9905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A169" s="25" t="s">
         <v>248</v>
       </c>
@@ -9943,7 +9946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A170" s="25" t="s">
         <v>249</v>
       </c>
@@ -9984,7 +9987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A171" s="25" t="s">
         <v>79</v>
       </c>
@@ -10025,7 +10028,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="172" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A172" s="31" t="s">
         <v>80</v>
       </c>
@@ -10066,7 +10069,7 @@
         <v>2.0000000000000001E-9</v>
       </c>
     </row>
-    <row r="173" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A173" s="31" t="s">
         <v>250</v>
       </c>
@@ -10107,7 +10110,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="174" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A174" s="31" t="s">
         <v>251</v>
       </c>
@@ -10148,7 +10151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A175" s="31" t="s">
         <v>252</v>
       </c>
@@ -10189,7 +10192,7 @@
         <v>3.98</v>
       </c>
     </row>
-    <row r="176" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A176" s="31" t="s">
         <v>253</v>
       </c>
@@ -10230,7 +10233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A177" s="31" t="s">
         <v>81</v>
       </c>
@@ -10271,7 +10274,7 @@
         <v>1.6666666666666666E-4</v>
       </c>
     </row>
-    <row r="178" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A178" s="11" t="s">
         <v>254</v>
       </c>
@@ -10312,7 +10315,7 @@
         <v>1E-8</v>
       </c>
     </row>
-    <row r="179" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A179" s="11" t="s">
         <v>255</v>
       </c>
@@ -10353,7 +10356,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="180" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A180" s="11" t="s">
         <v>256</v>
       </c>
@@ -10394,7 +10397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A181" s="11" t="s">
         <v>257</v>
       </c>
@@ -10435,7 +10438,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="182" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A182" s="11" t="s">
         <v>258</v>
       </c>
@@ -10476,7 +10479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A183" s="11" t="s">
         <v>259</v>
       </c>
@@ -10517,7 +10520,7 @@
         <v>8.3333333333333331E-5</v>
       </c>
     </row>
-    <row r="184" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A184" s="11" t="s">
         <v>260</v>
       </c>
@@ -10558,7 +10561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A185" s="27" t="s">
         <v>261</v>
       </c>
@@ -10599,7 +10602,7 @@
         <v>2.3533050791148899E-8</v>
       </c>
     </row>
-    <row r="186" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A186" s="27" t="s">
         <v>262</v>
       </c>
@@ -10640,7 +10643,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="187" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A187" s="27" t="s">
         <v>263</v>
       </c>
@@ -10681,7 +10684,7 @@
         <v>-0.187</v>
       </c>
     </row>
-    <row r="188" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A188" s="27" t="s">
         <v>264</v>
       </c>
@@ -10722,7 +10725,7 @@
         <v>2.48</v>
       </c>
     </row>
-    <row r="189" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A189" s="27" t="s">
         <v>265</v>
       </c>
@@ -10763,7 +10766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A190" s="27" t="s">
         <v>266</v>
       </c>
@@ -10804,7 +10807,7 @@
         <v>6.1060227588121015E-4</v>
       </c>
     </row>
-    <row r="191" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A191" s="23" t="s">
         <v>267</v>
       </c>
@@ -10845,7 +10848,7 @@
         <v>3.9999999999999998E-7</v>
       </c>
     </row>
-    <row r="192" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A192" s="23" t="s">
         <v>268</v>
       </c>
@@ -10886,7 +10889,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="193" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A193" s="23" t="s">
         <v>269</v>
       </c>
@@ -10927,7 +10930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A194" s="23" t="s">
         <v>270</v>
       </c>
@@ -10968,7 +10971,7 @@
         <v>3.98</v>
       </c>
     </row>
-    <row r="195" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A195" s="23" t="s">
         <v>271</v>
       </c>
@@ -11009,7 +11012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A196" s="23" t="s">
         <v>272</v>
       </c>
@@ -11050,7 +11053,7 @@
         <v>8.3333333333333331E-5</v>
       </c>
     </row>
-    <row r="197" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A197" s="7" t="s">
         <v>273</v>
       </c>
@@ -11091,7 +11094,7 @@
         <v>3.9999999999999998E-7</v>
       </c>
     </row>
-    <row r="198" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A198" s="7" t="s">
         <v>274</v>
       </c>
@@ -11132,7 +11135,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="199" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A199" s="7" t="s">
         <v>275</v>
       </c>
@@ -11173,7 +11176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A200" s="7" t="s">
         <v>276</v>
       </c>
@@ -11214,7 +11217,7 @@
         <v>3.98</v>
       </c>
     </row>
-    <row r="201" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A201" s="7" t="s">
         <v>277</v>
       </c>
@@ -11255,7 +11258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A202" s="7" t="s">
         <v>278</v>
       </c>
@@ -11296,7 +11299,7 @@
         <v>8.3333333333333331E-5</v>
       </c>
     </row>
-    <row r="203" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A203" s="29" t="s">
         <v>279</v>
       </c>
@@ -11337,7 +11340,7 @@
         <v>1.9999999999999999E-7</v>
       </c>
     </row>
-    <row r="204" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A204" s="29" t="s">
         <v>280</v>
       </c>
@@ -11378,7 +11381,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="205" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A205" s="29" t="s">
         <v>281</v>
       </c>
@@ -11419,7 +11422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A206" s="29" t="s">
         <v>282</v>
       </c>
@@ -11460,7 +11463,7 @@
         <v>3.98</v>
       </c>
     </row>
-    <row r="207" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A207" s="29" t="s">
         <v>283</v>
       </c>
@@ -11501,7 +11504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A208" s="29" t="s">
         <v>284</v>
       </c>
@@ -11542,7 +11545,7 @@
         <v>8.3333333333333331E-5</v>
       </c>
     </row>
-    <row r="209" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A209" s="90" t="s">
         <v>362</v>
       </c>
@@ -11583,7 +11586,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="210" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A210" s="2" t="s">
         <v>495</v>
       </c>
@@ -11624,7 +11627,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="211" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A211" s="2" t="s">
         <v>499</v>
       </c>
@@ -11665,7 +11668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A212" s="2" t="s">
         <v>522</v>
       </c>
@@ -11710,7 +11713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A213" s="2" t="s">
         <v>513</v>
       </c>
@@ -11751,7 +11754,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="214" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A214" s="2" t="s">
         <v>514</v>
       </c>
@@ -11792,7 +11795,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="215" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A215" s="2" t="s">
         <v>515</v>
       </c>
@@ -11833,7 +11836,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="216" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A216" s="2" t="s">
         <v>516</v>
       </c>
@@ -11874,7 +11877,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="217" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A217" s="2" t="s">
         <v>526</v>
       </c>
@@ -11915,7 +11918,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="218" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A218" s="2" t="s">
         <v>528</v>
       </c>
@@ -11939,20 +11942,20 @@
         <v>1.2499999999999999E-6</v>
       </c>
       <c r="H218" s="99">
-        <f>1250*0.000001/5</f>
-        <v>2.5000000000000001E-4</v>
+        <f>1.25*0.000001</f>
+        <v>1.2499999999999999E-6</v>
       </c>
       <c r="I218" s="99">
         <f>H218</f>
-        <v>2.5000000000000001E-4</v>
+        <v>1.2499999999999999E-6</v>
       </c>
       <c r="J218" s="99">
         <f t="shared" ref="J218:K218" si="2">I218</f>
-        <v>2.5000000000000001E-4</v>
+        <v>1.2499999999999999E-6</v>
       </c>
       <c r="K218" s="99">
         <f t="shared" si="2"/>
-        <v>2.5000000000000001E-4</v>
+        <v>1.2499999999999999E-6</v>
       </c>
       <c r="L218" s="99">
         <v>2.5000000000000001E-4</v>
@@ -11961,7 +11964,7 @@
         <v>2.5000000000000001E-4</v>
       </c>
     </row>
-    <row r="219" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A219" s="2" t="s">
         <v>531</v>
       </c>
@@ -12002,7 +12005,7 @@
         <v>9.9999999999999994E-12</v>
       </c>
     </row>
-    <row r="220" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A220" s="2" t="s">
         <v>534</v>
       </c>
@@ -12043,7 +12046,7 @@
         <v>2.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="221" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A221" s="2" t="s">
         <v>550</v>
       </c>
@@ -12069,7 +12072,7 @@
         <v>2.4999999999999998E-12</v>
       </c>
     </row>
-    <row r="222" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A222" s="2" t="s">
         <v>551</v>
       </c>
@@ -12095,7 +12098,7 @@
         <v>1.2E-8</v>
       </c>
     </row>
-    <row r="223" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A223" s="2" t="s">
         <v>552</v>
       </c>
@@ -12121,7 +12124,7 @@
         <v>9.9999999999999995E-8</v>
       </c>
     </row>
-    <row r="224" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A224" s="2" t="s">
         <v>553</v>
       </c>
@@ -12149,7 +12152,7 @@
         <v>2.0000000000000002E-5</v>
       </c>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A225" s="2" t="s">
         <v>531</v>
       </c>
@@ -12177,7 +12180,7 @@
         <v>9.9999999999999994E-12</v>
       </c>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A226" s="2" t="s">
         <v>554</v>
       </c>
@@ -12205,7 +12208,7 @@
         <v>1E-10</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A227" s="2" t="s">
         <v>555</v>
       </c>
@@ -12233,7 +12236,7 @@
         <v>0.10886399999999999</v>
       </c>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A228" s="2" t="s">
         <v>556</v>
       </c>
@@ -12259,7 +12262,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A229" s="2" t="s">
         <v>557</v>
       </c>
@@ -12285,7 +12288,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A230" s="2" t="s">
         <v>558</v>
       </c>
@@ -12313,7 +12316,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="231" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A231" s="2" t="s">
         <v>559</v>
       </c>
@@ -12339,7 +12342,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="232" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A232" s="2" t="s">
         <v>560</v>
       </c>
@@ -12363,11 +12366,60 @@
       </c>
       <c r="H232" s="98">
         <v>1.0000000000000001E-5</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H233" s="1" t="s">
+        <v>577</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H127:K128">
     <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H129:M129">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H130:M130">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -12542,50 +12594,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H130:M130">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H129:M129">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -12594,13 +12602,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C169"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="35.7109375" customWidth="1"/>
-    <col min="3" max="3" width="49.5703125" customWidth="1"/>
+    <col min="1" max="2" width="35.6640625" customWidth="1"/>
+    <col min="3" max="3" width="49.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>286</v>
       </c>
@@ -12611,7 +12619,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>206</v>
       </c>
@@ -12623,7 +12631,7 @@
         <v>pi</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -12635,7 +12643,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -12647,7 +12655,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>207</v>
       </c>
@@ -12659,7 +12667,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -12671,7 +12679,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -12683,7 +12691,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -12695,7 +12703,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>49</v>
       </c>
@@ -12707,7 +12715,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -12719,7 +12727,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -12731,7 +12739,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>46</v>
       </c>
@@ -12743,7 +12751,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -12755,7 +12763,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>91</v>
       </c>
@@ -12767,7 +12775,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -12779,7 +12787,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>208</v>
       </c>
@@ -12791,7 +12799,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -12803,7 +12811,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>50</v>
       </c>
@@ -12815,7 +12823,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>205</v>
       </c>
@@ -12827,7 +12835,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>51</v>
       </c>
@@ -12839,7 +12847,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>52</v>
       </c>
@@ -12851,7 +12859,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -12863,7 +12871,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>55</v>
       </c>
@@ -12875,7 +12883,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -12887,7 +12895,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>60</v>
       </c>
@@ -12899,7 +12907,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>209</v>
       </c>
@@ -12911,7 +12919,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>210</v>
       </c>
@@ -12923,7 +12931,7 @@
         <v>root_growth_T_ref</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>211</v>
       </c>
@@ -12935,7 +12943,7 @@
         <v>root_growth_A</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>212</v>
       </c>
@@ -12947,7 +12955,7 @@
         <v>root_growth_B</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>213</v>
       </c>
@@ -12959,7 +12967,7 @@
         <v>root_growth_C</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>214</v>
       </c>
@@ -12971,7 +12979,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>215</v>
       </c>
@@ -12983,7 +12991,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>216</v>
       </c>
@@ -12995,7 +13003,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>217</v>
       </c>
@@ -13007,7 +13015,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>218</v>
       </c>
@@ -13019,7 +13027,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>61</v>
       </c>
@@ -13031,7 +13039,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>75</v>
       </c>
@@ -13043,7 +13051,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>219</v>
       </c>
@@ -13055,7 +13063,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>220</v>
       </c>
@@ -13067,7 +13075,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>221</v>
       </c>
@@ -13079,7 +13087,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>222</v>
       </c>
@@ -13091,7 +13099,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>76</v>
       </c>
@@ -13103,7 +13111,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>223</v>
       </c>
@@ -13115,7 +13123,7 @@
         <v>expected_C_sucrose_root</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>224</v>
       </c>
@@ -13127,7 +13135,7 @@
         <v>expected_C_hexose_root</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>225</v>
       </c>
@@ -13139,7 +13147,7 @@
         <v>expected_C_hexose_soil</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>226</v>
       </c>
@@ -13151,7 +13159,7 @@
         <v>expected_C_hexose_reserve</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>65</v>
       </c>
@@ -13163,7 +13171,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>77</v>
       </c>
@@ -13175,7 +13183,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>227</v>
       </c>
@@ -13187,7 +13195,7 @@
         <v>surfacic_unloading_rate_reference</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>228</v>
       </c>
@@ -13199,7 +13207,7 @@
         <v>surfacic_unloading_rate_primordium</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>66</v>
       </c>
@@ -13211,7 +13219,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>229</v>
       </c>
@@ -13223,7 +13231,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>230</v>
       </c>
@@ -13235,7 +13243,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>231</v>
       </c>
@@ -13247,7 +13255,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>232</v>
       </c>
@@ -13259,7 +13267,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>68</v>
       </c>
@@ -13271,7 +13279,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>233</v>
       </c>
@@ -13283,7 +13291,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>234</v>
       </c>
@@ -13295,7 +13303,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>235</v>
       </c>
@@ -13307,7 +13315,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>236</v>
       </c>
@@ -13319,7 +13327,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -13331,7 +13339,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>70</v>
       </c>
@@ -13343,7 +13351,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>69</v>
       </c>
@@ -13355,7 +13363,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>57</v>
       </c>
@@ -13367,7 +13375,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>56</v>
       </c>
@@ -13379,7 +13387,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>58</v>
       </c>
@@ -13391,7 +13399,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>71</v>
       </c>
@@ -13403,7 +13411,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>237</v>
       </c>
@@ -13415,7 +13423,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>238</v>
       </c>
@@ -13427,7 +13435,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>239</v>
       </c>
@@ -13439,7 +13447,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>240</v>
       </c>
@@ -13451,7 +13459,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>72</v>
       </c>
@@ -13463,7 +13471,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>73</v>
       </c>
@@ -13475,7 +13483,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>241</v>
       </c>
@@ -13487,7 +13495,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>242</v>
       </c>
@@ -13499,7 +13507,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>243</v>
       </c>
@@ -13511,7 +13519,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>244</v>
       </c>
@@ -13523,7 +13531,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>74</v>
       </c>
@@ -13535,7 +13543,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>245</v>
       </c>
@@ -13547,7 +13555,7 @@
         <v>expected_exudation_efflux</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>78</v>
       </c>
@@ -13559,7 +13567,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>246</v>
       </c>
@@ -13571,7 +13579,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>247</v>
       </c>
@@ -13583,7 +13591,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>248</v>
       </c>
@@ -13595,7 +13603,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>249</v>
       </c>
@@ -13607,7 +13615,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>79</v>
       </c>
@@ -13619,7 +13627,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>80</v>
       </c>
@@ -13631,7 +13639,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>250</v>
       </c>
@@ -13643,7 +13651,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>251</v>
       </c>
@@ -13655,7 +13663,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>252</v>
       </c>
@@ -13667,7 +13675,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>253</v>
       </c>
@@ -13679,7 +13687,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>81</v>
       </c>
@@ -13691,7 +13699,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>254</v>
       </c>
@@ -13703,7 +13711,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>255</v>
       </c>
@@ -13715,7 +13723,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>256</v>
       </c>
@@ -13727,7 +13735,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>257</v>
       </c>
@@ -13739,7 +13747,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>258</v>
       </c>
@@ -13751,7 +13759,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>259</v>
       </c>
@@ -13763,7 +13771,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>260</v>
       </c>
@@ -13775,7 +13783,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>261</v>
       </c>
@@ -13787,7 +13795,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>262</v>
       </c>
@@ -13799,7 +13807,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>263</v>
       </c>
@@ -13811,7 +13819,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>264</v>
       </c>
@@ -13823,7 +13831,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>265</v>
       </c>
@@ -13835,7 +13843,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>266</v>
       </c>
@@ -13847,7 +13855,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>267</v>
       </c>
@@ -13859,7 +13867,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>268</v>
       </c>
@@ -13871,7 +13879,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>269</v>
       </c>
@@ -13883,7 +13891,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>270</v>
       </c>
@@ -13895,7 +13903,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>271</v>
       </c>
@@ -13907,7 +13915,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>272</v>
       </c>
@@ -13919,7 +13927,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>273</v>
       </c>
@@ -13931,7 +13939,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>274</v>
       </c>
@@ -13943,7 +13951,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>275</v>
       </c>
@@ -13955,7 +13963,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>276</v>
       </c>
@@ -13967,7 +13975,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>277</v>
       </c>
@@ -13979,7 +13987,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>278</v>
       </c>
@@ -13991,7 +13999,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>279</v>
       </c>
@@ -14003,7 +14011,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>280</v>
       </c>
@@ -14015,7 +14023,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>281</v>
       </c>
@@ -14027,7 +14035,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>282</v>
       </c>
@@ -14039,7 +14047,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>283</v>
       </c>
@@ -14051,7 +14059,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>284</v>
       </c>
@@ -14063,7 +14071,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>59</v>
       </c>
@@ -14075,7 +14083,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>62</v>
       </c>
@@ -14087,7 +14095,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>64</v>
       </c>
@@ -14099,7 +14107,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>63</v>
       </c>
@@ -14111,7 +14119,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>82</v>
       </c>
@@ -14123,7 +14131,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>83</v>
       </c>
@@ -14135,7 +14143,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>85</v>
       </c>
@@ -14147,7 +14155,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>84</v>
       </c>
@@ -14159,7 +14167,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>2</v>
       </c>
@@ -14171,7 +14179,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>4</v>
       </c>
@@ -14183,7 +14191,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>5</v>
       </c>
@@ -14195,7 +14203,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>20</v>
       </c>
@@ -14207,7 +14215,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>0</v>
       </c>
@@ -14219,7 +14227,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>1</v>
       </c>
@@ -14231,7 +14239,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>6</v>
       </c>
@@ -14243,7 +14251,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>7</v>
       </c>
@@ -14255,7 +14263,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>8</v>
       </c>
@@ -14267,7 +14275,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>9</v>
       </c>
@@ -14279,7 +14287,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>10</v>
       </c>
@@ -14291,7 +14299,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>11</v>
       </c>
@@ -14303,7 +14311,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>12</v>
       </c>
@@ -14315,7 +14323,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>13</v>
       </c>
@@ -14327,7 +14335,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>14</v>
       </c>
@@ -14339,7 +14347,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>15</v>
       </c>
@@ -14351,7 +14359,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>16</v>
       </c>
@@ -14363,7 +14371,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>17</v>
       </c>
@@ -14375,7 +14383,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>18</v>
       </c>
@@ -14387,7 +14395,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>19</v>
       </c>
@@ -14399,7 +14407,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>21</v>
       </c>
@@ -14411,7 +14419,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>22</v>
       </c>
@@ -14423,7 +14431,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>23</v>
       </c>
@@ -14435,7 +14443,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>24</v>
       </c>
@@ -14447,7 +14455,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>25</v>
       </c>
@@ -14459,7 +14467,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>26</v>
       </c>
@@ -14471,7 +14479,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>27</v>
       </c>
@@ -14483,7 +14491,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>28</v>
       </c>
@@ -14492,7 +14500,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>29</v>
       </c>
@@ -14501,7 +14509,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>30</v>
       </c>
@@ -14510,7 +14518,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>31</v>
       </c>
@@ -14519,7 +14527,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>32</v>
       </c>
@@ -14528,7 +14536,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>33</v>
       </c>
@@ -14537,7 +14545,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>34</v>
       </c>
@@ -14546,7 +14554,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>35</v>
       </c>
@@ -14555,7 +14563,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>36</v>
       </c>
@@ -14564,7 +14572,7 @@
         <v/>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>37</v>
       </c>
@@ -14573,7 +14581,7 @@
         <v/>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>38</v>
       </c>
@@ -14582,7 +14590,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>362</v>
       </c>

</xml_diff>